<commit_message>
Fixed Tomatometer Icon issue
</commit_message>
<xml_diff>
--- a/MovieListBoxOffice_WithTomatometer.xlsx
+++ b/MovieListBoxOffice_WithTomatometer.xlsx
@@ -1265,7 +1265,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1573,7 @@
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -1727,7 +1727,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1804,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2035,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -2805,7 +2805,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2882,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -2959,7 +2959,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3036,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -3190,7 +3190,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3498,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3806,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -3960,7 +3960,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -4422,7 +4422,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -4807,7 +4807,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -4884,7 +4884,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -5115,7 +5115,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -5180,9 +5180,21 @@
       <c r="N62" t="b">
         <v>0</v>
       </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>91%</t>
+        </is>
+      </c>
+      <c r="P62" t="inlineStr">
+        <is>
+          <t>278 Reviews</t>
+        </is>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -5873,7 +5885,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -6027,7 +6039,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -6104,7 +6116,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -6258,7 +6270,7 @@
       </c>
       <c r="Q76" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6347,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -6489,7 +6501,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -6720,7 +6732,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -6797,7 +6809,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -6874,7 +6886,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7028,7 +7040,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7182,7 +7194,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7247,21 +7259,9 @@
       <c r="N89" t="b">
         <v>0</v>
       </c>
-      <c r="O89" t="inlineStr">
-        <is>
-          <t>17%</t>
-        </is>
-      </c>
-      <c r="P89" t="inlineStr">
-        <is>
-          <t>138 Reviews</t>
-        </is>
-      </c>
-      <c r="Q89" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
+      <c r="O89" t="inlineStr"/>
+      <c r="P89" t="inlineStr"/>
+      <c r="Q89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -7336,7 +7336,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7490,7 +7490,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7567,7 +7567,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7644,7 +7644,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7721,7 +7721,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7875,7 +7875,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -7952,7 +7952,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -8029,7 +8029,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -8183,7 +8183,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -8260,7 +8260,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -8568,7 +8568,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -8876,7 +8876,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -9030,7 +9030,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -9184,7 +9184,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -9338,7 +9338,7 @@
       </c>
       <c r="Q116" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -9415,7 +9415,7 @@
       </c>
       <c r="Q117" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -9569,7 +9569,7 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -9646,7 +9646,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -9723,7 +9723,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -9877,7 +9877,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -10031,7 +10031,7 @@
       </c>
       <c r="Q125" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -10108,7 +10108,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -10647,7 +10647,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -10801,7 +10801,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -10878,7 +10878,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -10955,7 +10955,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -11174,7 +11174,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -11251,7 +11251,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -11482,7 +11482,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -11636,7 +11636,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -11713,7 +11713,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -11790,7 +11790,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -11867,7 +11867,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -11944,7 +11944,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -12175,7 +12175,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -12252,7 +12252,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -12406,7 +12406,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -12702,7 +12702,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -13419,7 +13419,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -13496,7 +13496,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -13573,7 +13573,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -13946,7 +13946,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -14100,7 +14100,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -14408,7 +14408,7 @@
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -14562,7 +14562,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -14716,7 +14716,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -14870,7 +14870,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -15101,7 +15101,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -15332,7 +15332,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -15563,7 +15563,7 @@
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -15640,7 +15640,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -15717,7 +15717,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -15794,7 +15794,7 @@
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -15948,7 +15948,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -16025,7 +16025,7 @@
       </c>
       <c r="Q43" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -16410,7 +16410,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -16564,7 +16564,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -16641,7 +16641,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -16718,7 +16718,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -16795,7 +16795,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -16949,7 +16949,7 @@
       </c>
       <c r="Q55" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -17103,7 +17103,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -17257,7 +17257,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -17565,7 +17565,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -17642,7 +17642,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -17796,7 +17796,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -17873,7 +17873,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -18104,7 +18104,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -18181,7 +18181,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -18258,7 +18258,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -18489,7 +18489,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -18720,7 +18720,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -18874,7 +18874,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -18951,7 +18951,7 @@
       </c>
       <c r="Q81" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -19105,7 +19105,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -19259,7 +19259,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -19336,7 +19336,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -19413,7 +19413,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -19567,7 +19567,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -19644,7 +19644,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -20029,7 +20029,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -20568,7 +20568,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -20645,7 +20645,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -20799,7 +20799,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -21030,7 +21030,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -21107,7 +21107,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -21184,7 +21184,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -21338,7 +21338,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -21415,7 +21415,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -21492,7 +21492,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -21800,7 +21800,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -22262,7 +22262,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -22416,7 +22416,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -22570,7 +22570,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -22801,7 +22801,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -22878,7 +22878,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -23109,7 +23109,7 @@
       </c>
       <c r="Q135" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -23263,7 +23263,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -23340,7 +23340,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -23494,7 +23494,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -23636,7 +23636,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -23713,7 +23713,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -23790,7 +23790,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -24021,7 +24021,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -24098,7 +24098,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -24394,7 +24394,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -24471,7 +24471,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -24548,7 +24548,7 @@
       </c>
       <c r="Q154" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -24779,7 +24779,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -25010,7 +25010,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -25152,7 +25152,7 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -25229,7 +25229,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -25306,7 +25306,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -25448,7 +25448,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -26179,7 +26179,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -26337,7 +26337,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -26969,7 +26969,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -27048,7 +27048,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -27127,7 +27127,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -27680,7 +27680,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -27838,7 +27838,7 @@
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -27996,7 +27996,7 @@
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -28075,7 +28075,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -28312,7 +28312,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -28549,7 +28549,7 @@
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -28628,7 +28628,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -28786,7 +28786,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -28865,7 +28865,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -29102,7 +29102,7 @@
       </c>
       <c r="Q45" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -29181,7 +29181,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -29339,7 +29339,7 @@
       </c>
       <c r="Q48" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -29418,7 +29418,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -29497,7 +29497,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -29813,7 +29813,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30050,7 +30050,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30208,7 +30208,7 @@
       </c>
       <c r="Q59" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30287,7 +30287,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30366,7 +30366,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30445,7 +30445,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30524,7 +30524,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30603,7 +30603,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30682,7 +30682,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30761,7 +30761,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30919,7 +30919,7 @@
       </c>
       <c r="Q68" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -30998,7 +30998,7 @@
       </c>
       <c r="Q69" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -31156,7 +31156,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -31235,7 +31235,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -31314,7 +31314,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -31472,7 +31472,7 @@
       </c>
       <c r="Q75" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -31630,7 +31630,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -31709,7 +31709,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -31788,7 +31788,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -31867,7 +31867,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -32025,7 +32025,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -32104,7 +32104,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -32183,7 +32183,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -32341,7 +32341,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -32578,7 +32578,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -32657,7 +32657,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -32736,7 +32736,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -32973,7 +32973,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -33052,7 +33052,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -33210,7 +33210,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -33289,7 +33289,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -33593,7 +33593,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -33672,7 +33672,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -33751,7 +33751,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -34067,7 +34067,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -34146,7 +34146,7 @@
       </c>
       <c r="Q109" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -34225,7 +34225,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -34462,7 +34462,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35015,7 +35015,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35094,7 +35094,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35252,7 +35252,7 @@
       </c>
       <c r="Q123" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35331,7 +35331,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35568,7 +35568,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35726,7 +35726,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35805,7 +35805,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35884,7 +35884,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -35963,7 +35963,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -36042,7 +36042,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -36279,7 +36279,7 @@
       </c>
       <c r="Q136" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -36358,7 +36358,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -36437,7 +36437,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -36516,7 +36516,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -36595,7 +36595,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -36674,7 +36674,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -36911,7 +36911,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -37215,7 +37215,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -37294,7 +37294,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -37531,7 +37531,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -37811,7 +37811,7 @@
       </c>
       <c r="Q156" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -37890,7 +37890,7 @@
       </c>
       <c r="Q157" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -37969,7 +37969,7 @@
       </c>
       <c r="Q158" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -38048,7 +38048,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -38127,7 +38127,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -38431,7 +38431,7 @@
       </c>
       <c r="Q164" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -38589,7 +38589,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -38948,7 +38948,7 @@
       </c>
       <c r="Q171" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -39791,7 +39791,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -39949,7 +39949,7 @@
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -40107,7 +40107,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -40423,7 +40423,7 @@
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -40976,7 +40976,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -41134,7 +41134,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -41529,7 +41529,7 @@
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -41845,7 +41845,7 @@
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -41924,7 +41924,7 @@
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -42003,7 +42003,7 @@
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -42082,7 +42082,7 @@
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -42556,7 +42556,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -42635,7 +42635,7 @@
       </c>
       <c r="Q42" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -42939,7 +42939,7 @@
       </c>
       <c r="Q46" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -43018,7 +43018,7 @@
       </c>
       <c r="Q47" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -43255,7 +43255,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -43334,7 +43334,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -43413,7 +43413,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -43492,7 +43492,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -43571,7 +43571,7 @@
       </c>
       <c r="Q54" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -43729,7 +43729,7 @@
       </c>
       <c r="Q56" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -43808,7 +43808,7 @@
       </c>
       <c r="Q57" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44112,7 +44112,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44191,7 +44191,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44270,7 +44270,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44349,7 +44349,7 @@
       </c>
       <c r="Q64" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44428,7 +44428,7 @@
       </c>
       <c r="Q65" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44507,7 +44507,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44586,7 +44586,7 @@
       </c>
       <c r="Q67" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44653,9 +44653,21 @@
       <c r="N68" t="b">
         <v>0</v>
       </c>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>87%</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr">
+        <is>
+          <t>463 Reviews</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -44811,7 +44823,7 @@
       </c>
       <c r="Q70" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -44890,7 +44902,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -45127,7 +45139,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -45364,7 +45376,7 @@
       </c>
       <c r="Q77" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -45443,7 +45455,7 @@
       </c>
       <c r="Q78" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -45522,7 +45534,7 @@
       </c>
       <c r="Q79" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -45601,7 +45613,7 @@
       </c>
       <c r="Q80" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -45747,7 +45759,7 @@
       </c>
       <c r="Q82" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -45905,7 +45917,7 @@
       </c>
       <c r="Q84" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -45984,7 +45996,7 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -46374,7 +46386,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>88 Reviews</t>
+          <t>90 Reviews</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr">
@@ -46458,7 +46470,7 @@
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -46537,7 +46549,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -46616,7 +46628,7 @@
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -47169,7 +47181,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -47248,7 +47260,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -47327,7 +47339,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -47643,7 +47655,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -47722,7 +47734,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -47801,7 +47813,7 @@
       </c>
       <c r="Q108" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -48038,7 +48050,7 @@
       </c>
       <c r="Q111" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -48275,7 +48287,7 @@
       </c>
       <c r="Q114" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -48591,7 +48603,7 @@
       </c>
       <c r="Q118" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -48670,7 +48682,7 @@
       </c>
       <c r="Q119" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -48749,7 +48761,7 @@
       </c>
       <c r="Q120" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -48828,7 +48840,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -48907,7 +48919,7 @@
       </c>
       <c r="Q122" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -49065,7 +49077,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -49302,7 +49314,7 @@
       </c>
       <c r="Q127" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -49381,7 +49393,7 @@
       </c>
       <c r="Q128" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -49460,7 +49472,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -49539,7 +49551,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -49697,7 +49709,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -50171,7 +50183,7 @@
       </c>
       <c r="Q138" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -50329,7 +50341,7 @@
       </c>
       <c r="Q140" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -50408,7 +50420,7 @@
       </c>
       <c r="Q141" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -50566,7 +50578,7 @@
       </c>
       <c r="Q143" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -50645,7 +50657,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -50882,7 +50894,7 @@
       </c>
       <c r="Q147" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -50961,7 +50973,7 @@
       </c>
       <c r="Q148" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -51040,7 +51052,7 @@
       </c>
       <c r="Q149" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -51119,7 +51131,7 @@
       </c>
       <c r="Q150" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -51277,7 +51289,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -51356,7 +51368,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -51502,7 +51514,7 @@
       </c>
       <c r="Q155" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -51818,7 +51830,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -51897,7 +51909,7 @@
       </c>
       <c r="Q160" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -52122,7 +52134,7 @@
       </c>
       <c r="Q163" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -52347,7 +52359,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -52493,7 +52505,7 @@
       </c>
       <c r="Q168" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -52785,7 +52797,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -53077,7 +53089,7 @@
       </c>
       <c r="Q176" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -53953,7 +53965,7 @@
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -54032,7 +54044,7 @@
       </c>
       <c r="Q189" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -54817,7 +54829,7 @@
       </c>
       <c r="Q200" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -55155,7 +55167,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -55234,7 +55246,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -55629,7 +55641,7 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -55708,7 +55720,7 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -55945,7 +55957,7 @@
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -56735,7 +56747,7 @@
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -56814,7 +56826,7 @@
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -56972,7 +56984,7 @@
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -57051,7 +57063,7 @@
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -57288,7 +57300,7 @@
       </c>
       <c r="Q30" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -57762,7 +57774,7 @@
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -57987,7 +57999,7 @@
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -58145,7 +58157,7 @@
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -58382,7 +58394,7 @@
       </c>
       <c r="Q44" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -58777,7 +58789,7 @@
       </c>
       <c r="Q49" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -58856,7 +58868,7 @@
       </c>
       <c r="Q50" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -58935,7 +58947,7 @@
       </c>
       <c r="Q51" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -59014,7 +59026,7 @@
       </c>
       <c r="Q52" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -59093,7 +59105,7 @@
       </c>
       <c r="Q53" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -59488,7 +59500,7 @@
       </c>
       <c r="Q58" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -59646,7 +59658,7 @@
       </c>
       <c r="Q60" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -59725,7 +59737,7 @@
       </c>
       <c r="Q61" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -59804,7 +59816,7 @@
       </c>
       <c r="Q62" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -59883,7 +59895,7 @@
       </c>
       <c r="Q63" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -60120,7 +60132,7 @@
       </c>
       <c r="Q66" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -60515,7 +60527,7 @@
       </c>
       <c r="Q71" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -60594,7 +60606,7 @@
       </c>
       <c r="Q72" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -60673,7 +60685,7 @@
       </c>
       <c r="Q73" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -60752,7 +60764,7 @@
       </c>
       <c r="Q74" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -61463,7 +61475,7 @@
       </c>
       <c r="Q83" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -61700,7 +61712,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -61779,7 +61791,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -61858,7 +61870,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -62174,7 +62186,7 @@
       </c>
       <c r="Q92" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -62332,7 +62344,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -62490,7 +62502,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -62569,7 +62581,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -62885,7 +62897,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -62964,7 +62976,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -63043,7 +63055,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -63201,7 +63213,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -63596,7 +63608,7 @@
       </c>
       <c r="Q110" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -63754,7 +63766,7 @@
       </c>
       <c r="Q112" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -63833,7 +63845,7 @@
       </c>
       <c r="Q113" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -64465,7 +64477,7 @@
       </c>
       <c r="Q121" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -64702,7 +64714,7 @@
       </c>
       <c r="Q124" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -64860,7 +64872,7 @@
       </c>
       <c r="Q126" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -65097,7 +65109,7 @@
       </c>
       <c r="Q129" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -65176,7 +65188,7 @@
       </c>
       <c r="Q130" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -65255,7 +65267,7 @@
       </c>
       <c r="Q131" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -65334,7 +65346,7 @@
       </c>
       <c r="Q132" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -65413,7 +65425,7 @@
       </c>
       <c r="Q133" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -65492,7 +65504,7 @@
       </c>
       <c r="Q134" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -65729,7 +65741,7 @@
       </c>
       <c r="Q137" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -65887,7 +65899,7 @@
       </c>
       <c r="Q139" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -66112,7 +66124,7 @@
       </c>
       <c r="Q142" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -66270,7 +66282,7 @@
       </c>
       <c r="Q144" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -66416,7 +66428,7 @@
       </c>
       <c r="Q146" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -66787,7 +66799,7 @@
       </c>
       <c r="Q151" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -66866,7 +66878,7 @@
       </c>
       <c r="Q152" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -66945,7 +66957,7 @@
       </c>
       <c r="Q153" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -67383,7 +67395,7 @@
       </c>
       <c r="Q159" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -67541,7 +67553,7 @@
       </c>
       <c r="Q161" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -67620,7 +67632,7 @@
       </c>
       <c r="Q162" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -67924,7 +67936,7 @@
       </c>
       <c r="Q166" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -68003,7 +68015,7 @@
       </c>
       <c r="Q167" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -68362,7 +68374,7 @@
       </c>
       <c r="Q172" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -69128,7 +69140,7 @@
       </c>
       <c r="Q182" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -69578,7 +69590,7 @@
       </c>
       <c r="Q188" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>
@@ -69973,7 +69985,7 @@
       </c>
       <c r="Q193" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Rotten</t>
         </is>
       </c>
     </row>

</xml_diff>